<commit_message>
fix pea add more countries
</commit_message>
<xml_diff>
--- a/data/raw/pea-tool.xlsx
+++ b/data/raw/pea-tool.xlsx
@@ -1,15 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29426"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F31D6075-2F6B-4D28-8D71-0E1233511904}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D1803ABD-E150-4DA6-9F7C-509739C8AE9E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="costs" sheetId="1" r:id="rId1"/>
-    <sheet name="GDP" sheetId="2" r:id="rId2"/>
+    <sheet name="calculating costs" sheetId="3" r:id="rId1"/>
+    <sheet name="costs" sheetId="1" r:id="rId2"/>
+    <sheet name="GDP" sheetId="2" r:id="rId3"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -32,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="227" uniqueCount="225">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="257" uniqueCount="239">
   <si>
     <t>env</t>
   </si>
@@ -691,9 +692,6 @@
     <t>-</t>
   </si>
   <si>
-    <t>cost_englishpounds_kg</t>
-  </si>
-  <si>
     <t>GDP_percapita_multiplier</t>
   </si>
   <si>
@@ -707,6 +705,51 @@
   </si>
   <si>
     <t>hum</t>
+  </si>
+  <si>
+    <t>Pesticides in sources of drinking water</t>
+  </si>
+  <si>
+    <t>Pollution incidents, fish deaths and monitoring costs</t>
+  </si>
+  <si>
+    <t>Biodiversity/wildlife losses</t>
+  </si>
+  <si>
+    <t>Cultural, landscape, toursim etc. (Hedgerows, dry stone walls, perception of spraying)</t>
+  </si>
+  <si>
+    <t>Bee colony losses</t>
+  </si>
+  <si>
+    <t>Acute effects of pesticides to human health</t>
+  </si>
+  <si>
+    <t>Total</t>
+  </si>
+  <si>
+    <t>cost_euros_kg</t>
+  </si>
+  <si>
+    <t>Cost application for moderate EIQ compound</t>
+  </si>
+  <si>
+    <t>Biodiversity / wildlife losses</t>
+  </si>
+  <si>
+    <t>Landscape / Cultural / tourism value</t>
+  </si>
+  <si>
+    <t>human</t>
+  </si>
+  <si>
+    <t>ecoterr</t>
+  </si>
+  <si>
+    <t>ecoaqu</t>
+  </si>
+  <si>
+    <t>From Adrian's sheet</t>
   </si>
 </sst>
 </file>
@@ -738,12 +781,92 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="9">
     <border>
       <left/>
       <right/>
       <top/>
       <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
       <diagonal/>
     </border>
   </borders>
@@ -753,8 +876,17 @@
     <xf numFmtId="164" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="4">
     <cellStyle name="Currency 2" xfId="2" xr:uid="{698E9EEC-4B79-4DA0-92EC-9F7370EA27DF}"/>
@@ -1091,11 +1223,11 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1881D26D-58E6-4B13-B3DA-2DFBBC0E86E2}">
-  <dimension ref="A1:B5"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FEDF9105-F914-4B19-9DAC-CD45C2DC44BB}">
+  <dimension ref="A1:I28"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="11.88671875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="62.77734375" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.3">
@@ -1103,12 +1235,12 @@
         <v>1</v>
       </c>
       <c r="B1" t="s">
-        <v>219</v>
+        <v>231</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
       <c r="B2">
         <v>8.4340999798966507</v>
@@ -1119,23 +1251,358 @@
         <v>0</v>
       </c>
       <c r="B3">
-        <v>2.1943095310840208</v>
+        <v>1.5793213512592963</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
-        <v>222</v>
+        <v>221</v>
       </c>
       <c r="B4">
-        <v>0.56791318969669236</v>
+        <v>1.2299763596494486</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
-        <v>223</v>
+        <v>222</v>
       </c>
       <c r="B5">
+        <v>0.9256913508458956</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="B6">
+        <f>SUM(B2:B5)</f>
+        <v>12.16908904165129</v>
+      </c>
+    </row>
+    <row r="9" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A9" t="s">
+        <v>224</v>
+      </c>
+      <c r="B9">
+        <v>7.7946313552285149</v>
+      </c>
+    </row>
+    <row r="10" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A10" t="s">
+        <v>225</v>
+      </c>
+      <c r="B10">
+        <v>1.2299763596494486</v>
+      </c>
+    </row>
+    <row r="11" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A11" t="s">
+        <v>226</v>
+      </c>
+      <c r="B11">
+        <v>0.71555632229840649</v>
+      </c>
+    </row>
+    <row r="12" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A12" t="s">
+        <v>227</v>
+      </c>
+      <c r="B12">
+        <v>1.5793213512592963</v>
+      </c>
+    </row>
+    <row r="13" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A13" t="s">
+        <v>228</v>
+      </c>
+      <c r="B13">
+        <v>0.21013502854748911</v>
+      </c>
+    </row>
+    <row r="14" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A14" t="s">
+        <v>229</v>
+      </c>
+      <c r="B14">
+        <v>0.63946862466813637</v>
+      </c>
+    </row>
+    <row r="15" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A15" t="s">
+        <v>230</v>
+      </c>
+      <c r="B15">
+        <v>12.169089041651292</v>
+      </c>
+    </row>
+    <row r="18" spans="1:9" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A18" t="s">
+        <v>238</v>
+      </c>
+    </row>
+    <row r="19" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A19" s="1"/>
+      <c r="B19" s="2" t="s">
+        <v>232</v>
+      </c>
+      <c r="C19" s="2" t="s">
+        <v>224</v>
+      </c>
+      <c r="D19" s="2" t="s">
+        <v>225</v>
+      </c>
+      <c r="E19" s="2" t="s">
+        <v>233</v>
+      </c>
+      <c r="F19" s="2" t="s">
+        <v>234</v>
+      </c>
+      <c r="G19" s="2" t="s">
+        <v>228</v>
+      </c>
+      <c r="H19" s="2" t="s">
+        <v>229</v>
+      </c>
+      <c r="I19" s="3" t="s">
+        <v>230</v>
+      </c>
+    </row>
+    <row r="20" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A20" s="4" t="s">
+        <v>235</v>
+      </c>
+      <c r="B20" s="5" t="s">
+        <v>235</v>
+      </c>
+      <c r="C20" s="5">
+        <v>7.7946313552285149</v>
+      </c>
+      <c r="D20" s="5">
+        <v>0</v>
+      </c>
+      <c r="E20" s="5">
+        <v>0</v>
+      </c>
+      <c r="F20" s="5">
+        <v>0</v>
+      </c>
+      <c r="G20" s="5">
+        <v>0</v>
+      </c>
+      <c r="H20" s="5">
+        <v>0.63946862466813637</v>
+      </c>
+      <c r="I20" s="6">
+        <v>8.4340999798966507</v>
+      </c>
+    </row>
+    <row r="21" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A21" s="4" t="s">
+        <v>0</v>
+      </c>
+      <c r="B21" s="5" t="s">
+        <v>0</v>
+      </c>
+      <c r="C21" s="5">
+        <v>0</v>
+      </c>
+      <c r="D21" s="5">
+        <v>0.61498817982472431</v>
+      </c>
+      <c r="E21" s="5">
+        <v>0</v>
+      </c>
+      <c r="F21" s="5">
+        <v>1.5793213512592963</v>
+      </c>
+      <c r="G21" s="5">
+        <v>0</v>
+      </c>
+      <c r="H21" s="5">
+        <v>0</v>
+      </c>
+      <c r="I21" s="6">
+        <v>2.1943095310840208</v>
+      </c>
+    </row>
+    <row r="22" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A22" s="4" t="s">
+        <v>236</v>
+      </c>
+      <c r="B22" s="5" t="s">
+        <v>236</v>
+      </c>
+      <c r="C22" s="5">
+        <v>0</v>
+      </c>
+      <c r="D22" s="5">
+        <v>0</v>
+      </c>
+      <c r="E22" s="5">
+        <v>0.35777816114920324</v>
+      </c>
+      <c r="F22" s="5">
+        <v>0</v>
+      </c>
+      <c r="G22" s="5">
+        <v>0.21013502854748911</v>
+      </c>
+      <c r="H22" s="5">
+        <v>0</v>
+      </c>
+      <c r="I22" s="6">
+        <v>0.56791318969669236</v>
+      </c>
+    </row>
+    <row r="23" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A23" s="4" t="s">
+        <v>237</v>
+      </c>
+      <c r="B23" s="5" t="s">
+        <v>237</v>
+      </c>
+      <c r="C23" s="5">
+        <v>0</v>
+      </c>
+      <c r="D23" s="5">
+        <v>0.61498817982472431</v>
+      </c>
+      <c r="E23" s="5">
+        <v>0.35777816114920324</v>
+      </c>
+      <c r="F23" s="5">
+        <v>0</v>
+      </c>
+      <c r="G23" s="5">
+        <v>0</v>
+      </c>
+      <c r="H23" s="5">
+        <v>0</v>
+      </c>
+      <c r="I23" s="6">
         <v>0.97276634097392756</v>
+      </c>
+    </row>
+    <row r="24" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A24" s="4"/>
+      <c r="B24" s="5"/>
+      <c r="C24" s="5">
+        <v>0</v>
+      </c>
+      <c r="D24" s="5">
+        <v>0</v>
+      </c>
+      <c r="E24" s="5">
+        <v>0</v>
+      </c>
+      <c r="F24" s="5">
+        <v>0</v>
+      </c>
+      <c r="G24" s="5">
+        <v>0</v>
+      </c>
+      <c r="H24" s="5">
+        <v>0</v>
+      </c>
+      <c r="I24" s="6">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="25" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A25" s="4"/>
+      <c r="B25" s="5"/>
+      <c r="C25" s="5">
+        <v>0</v>
+      </c>
+      <c r="D25" s="5">
+        <v>0</v>
+      </c>
+      <c r="E25" s="5">
+        <v>0</v>
+      </c>
+      <c r="F25" s="5">
+        <v>0</v>
+      </c>
+      <c r="G25" s="5">
+        <v>0</v>
+      </c>
+      <c r="H25" s="5">
+        <v>0</v>
+      </c>
+      <c r="I25" s="6">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="26" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A26" s="4"/>
+      <c r="B26" s="5"/>
+      <c r="C26" s="5">
+        <v>0</v>
+      </c>
+      <c r="D26" s="5">
+        <v>0</v>
+      </c>
+      <c r="E26" s="5">
+        <v>0</v>
+      </c>
+      <c r="F26" s="5">
+        <v>0</v>
+      </c>
+      <c r="G26" s="5">
+        <v>0</v>
+      </c>
+      <c r="H26" s="5">
+        <v>0</v>
+      </c>
+      <c r="I26" s="6">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="27" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A27" s="4"/>
+      <c r="B27" s="5"/>
+      <c r="C27" s="5">
+        <v>0</v>
+      </c>
+      <c r="D27" s="5">
+        <v>0</v>
+      </c>
+      <c r="E27" s="5">
+        <v>0</v>
+      </c>
+      <c r="F27" s="5">
+        <v>0</v>
+      </c>
+      <c r="G27" s="5">
+        <v>0</v>
+      </c>
+      <c r="H27" s="5">
+        <v>0</v>
+      </c>
+      <c r="I27" s="6">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="28" spans="1:9" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A28" s="7"/>
+      <c r="B28" s="8"/>
+      <c r="C28" s="8">
+        <v>7.7946313552285149</v>
+      </c>
+      <c r="D28" s="8">
+        <v>1.2299763596494486</v>
+      </c>
+      <c r="E28" s="8">
+        <v>0.71555632229840649</v>
+      </c>
+      <c r="F28" s="8">
+        <v>1.5793213512592963</v>
+      </c>
+      <c r="G28" s="8">
+        <v>0.21013502854748911</v>
+      </c>
+      <c r="H28" s="8">
+        <v>0.63946862466813637</v>
+      </c>
+      <c r="I28" s="9">
+        <v>12.16908904165129</v>
       </c>
     </row>
   </sheetData>
@@ -1145,6 +1612,60 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1881D26D-58E6-4B13-B3DA-2DFBBC0E86E2}">
+  <dimension ref="A1:B5"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="62.77734375" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A1" t="s">
+        <v>1</v>
+      </c>
+      <c r="B1" t="s">
+        <v>231</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A2" t="s">
+        <v>223</v>
+      </c>
+      <c r="B2">
+        <v>8.4340999798966507</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A3" t="s">
+        <v>0</v>
+      </c>
+      <c r="B3">
+        <v>2.1943095310840208</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A4" t="s">
+        <v>221</v>
+      </c>
+      <c r="B4">
+        <v>0.56791318969669236</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A5" t="s">
+        <v>222</v>
+      </c>
+      <c r="B5">
+        <v>0.97276634097392756</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2F7648E7-D030-4C64-9BB1-9DB3E6A86316}">
   <dimension ref="A1:C216"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
@@ -1159,10 +1680,10 @@
         <v>2</v>
       </c>
       <c r="B1" t="s">
+        <v>219</v>
+      </c>
+      <c r="C1" t="s">
         <v>220</v>
-      </c>
-      <c r="C1" t="s">
-        <v>221</v>
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.3">

</xml_diff>

<commit_message>
Add Jons cost things
</commit_message>
<xml_diff>
--- a/data/raw/pea-tool.xlsx
+++ b/data/raw/pea-tool.xlsx
@@ -1,9 +1,9 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
-  <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D1803ABD-E150-4DA6-9F7C-509739C8AE9E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
+  <workbookPr filterPrivacy="1" defaultThemeVersion="202300"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{82A5F708-278A-482B-A592-832E04B364CF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="257" uniqueCount="239">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="272" uniqueCount="240">
   <si>
     <t>env</t>
   </si>
@@ -750,6 +750,9 @@
   </si>
   <si>
     <t>From Adrian's sheet</t>
+  </si>
+  <si>
+    <t>0.5</t>
   </si>
 </sst>
 </file>
@@ -878,15 +881,33 @@
   </cellStyleXfs>
   <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="4">
     <cellStyle name="Currency 2" xfId="2" xr:uid="{698E9EEC-4B79-4DA0-92EC-9F7370EA27DF}"/>
@@ -1224,363 +1245,385 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FEDF9105-F914-4B19-9DAC-CD45C2DC44BB}">
-  <dimension ref="A1:I28"/>
+  <dimension ref="A1:J39"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="62.77734375" customWidth="1"/>
+    <col min="1" max="1" width="27.88671875" style="1" customWidth="1"/>
+    <col min="2" max="2" width="13.88671875" style="1" customWidth="1"/>
+    <col min="3" max="3" width="15.33203125" style="1" customWidth="1"/>
+    <col min="4" max="4" width="20.109375" style="1" customWidth="1"/>
+    <col min="5" max="5" width="16.44140625" style="1" customWidth="1"/>
+    <col min="6" max="6" width="8.88671875" style="1"/>
+    <col min="7" max="7" width="14.77734375" style="1" customWidth="1"/>
+    <col min="8" max="8" width="28.88671875" style="1" customWidth="1"/>
+    <col min="9" max="9" width="8.88671875" style="1"/>
+    <col min="10" max="10" width="11.5546875" style="1" bestFit="1" customWidth="1"/>
+    <col min="11" max="16384" width="8.88671875" style="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A1" t="s">
+      <c r="A1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B1" s="1" t="s">
         <v>231</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A2" t="s">
+      <c r="A2" s="1" t="s">
         <v>223</v>
       </c>
-      <c r="B2">
+      <c r="B2" s="1">
         <v>8.4340999798966507</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A3" t="s">
-        <v>0</v>
-      </c>
-      <c r="B3">
+      <c r="A3" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B3" s="1">
         <v>1.5793213512592963</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A4" t="s">
+      <c r="A4" s="1" t="s">
         <v>221</v>
       </c>
-      <c r="B4">
+      <c r="B4" s="1">
         <v>1.2299763596494486</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A5" t="s">
+      <c r="A5" s="1" t="s">
         <v>222</v>
       </c>
-      <c r="B5">
+      <c r="B5" s="1">
         <v>0.9256913508458956</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="B6">
+      <c r="B6" s="1">
         <f>SUM(B2:B5)</f>
         <v>12.16908904165129</v>
       </c>
     </row>
-    <row r="9" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A9" t="s">
+    <row r="9" spans="1:2" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A9" s="1" t="s">
         <v>224</v>
       </c>
-      <c r="B9">
+      <c r="B9" s="1">
         <v>7.7946313552285149</v>
       </c>
     </row>
-    <row r="10" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A10" t="s">
+    <row r="10" spans="1:2" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A10" s="1" t="s">
         <v>225</v>
       </c>
-      <c r="B10">
+      <c r="B10" s="1">
         <v>1.2299763596494486</v>
       </c>
     </row>
     <row r="11" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A11" t="s">
+      <c r="A11" s="1" t="s">
         <v>226</v>
       </c>
-      <c r="B11">
+      <c r="B11" s="1">
         <v>0.71555632229840649</v>
       </c>
     </row>
-    <row r="12" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A12" t="s">
+    <row r="12" spans="1:2" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="A12" s="1" t="s">
         <v>227</v>
       </c>
-      <c r="B12">
+      <c r="B12" s="1">
         <v>1.5793213512592963</v>
       </c>
     </row>
     <row r="13" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A13" t="s">
+      <c r="A13" s="1" t="s">
         <v>228</v>
       </c>
-      <c r="B13">
+      <c r="B13" s="1">
         <v>0.21013502854748911</v>
       </c>
     </row>
-    <row r="14" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A14" t="s">
+    <row r="14" spans="1:2" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A14" s="1" t="s">
         <v>229</v>
       </c>
-      <c r="B14">
+      <c r="B14" s="1">
         <v>0.63946862466813637</v>
       </c>
     </row>
     <row r="15" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A15" t="s">
+      <c r="A15" s="1" t="s">
         <v>230</v>
       </c>
-      <c r="B15">
+      <c r="B15" s="1">
         <v>12.169089041651292</v>
       </c>
     </row>
-    <row r="18" spans="1:9" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A18" t="s">
+    <row r="18" spans="1:10" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A18" s="1" t="s">
         <v>238</v>
       </c>
     </row>
-    <row r="19" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A19" s="1"/>
-      <c r="B19" s="2" t="s">
+    <row r="19" spans="1:10" ht="72" x14ac:dyDescent="0.3">
+      <c r="A19" s="2"/>
+      <c r="B19" s="3" t="s">
         <v>232</v>
       </c>
-      <c r="C19" s="2" t="s">
+      <c r="C19" s="3" t="s">
         <v>224</v>
       </c>
-      <c r="D19" s="2" t="s">
+      <c r="D19" s="3" t="s">
         <v>225</v>
       </c>
-      <c r="E19" s="2" t="s">
+      <c r="E19" s="3" t="s">
         <v>233</v>
       </c>
-      <c r="F19" s="2" t="s">
+      <c r="F19" s="3" t="s">
         <v>234</v>
       </c>
-      <c r="G19" s="2" t="s">
+      <c r="G19" s="3" t="s">
         <v>228</v>
       </c>
-      <c r="H19" s="2" t="s">
+      <c r="H19" s="3" t="s">
         <v>229</v>
       </c>
-      <c r="I19" s="3" t="s">
+      <c r="I19" s="4" t="s">
         <v>230</v>
       </c>
     </row>
-    <row r="20" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A20" s="4" t="s">
+    <row r="20" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A20" s="5" t="s">
         <v>235</v>
       </c>
-      <c r="B20" s="5" t="s">
+      <c r="B20" s="1" t="s">
         <v>235</v>
       </c>
-      <c r="C20" s="5">
+      <c r="C20" s="1">
         <v>7.7946313552285149</v>
       </c>
-      <c r="D20" s="5">
-        <v>0</v>
-      </c>
-      <c r="E20" s="5">
-        <v>0</v>
-      </c>
-      <c r="F20" s="5">
-        <v>0</v>
-      </c>
-      <c r="G20" s="5">
-        <v>0</v>
-      </c>
-      <c r="H20" s="5">
+      <c r="D20" s="1">
+        <v>0</v>
+      </c>
+      <c r="E20" s="1">
+        <v>0</v>
+      </c>
+      <c r="F20" s="1">
+        <v>0</v>
+      </c>
+      <c r="G20" s="1">
+        <v>0</v>
+      </c>
+      <c r="H20" s="1">
         <v>0.63946862466813637</v>
       </c>
       <c r="I20" s="6">
         <v>8.4340999798966507</v>
       </c>
-    </row>
-    <row r="21" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A21" s="4" t="s">
-        <v>0</v>
-      </c>
-      <c r="B21" s="5" t="s">
-        <v>0</v>
-      </c>
-      <c r="C21" s="5">
-        <v>0</v>
-      </c>
-      <c r="D21" s="5">
+      <c r="J20" s="1">
+        <f>I20/$I$28</f>
+        <v>0.69307570608031166</v>
+      </c>
+    </row>
+    <row r="21" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A21" s="5" t="s">
+        <v>0</v>
+      </c>
+      <c r="B21" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="C21" s="1">
+        <v>0</v>
+      </c>
+      <c r="D21" s="1">
         <v>0.61498817982472431</v>
       </c>
-      <c r="E21" s="5">
-        <v>0</v>
-      </c>
-      <c r="F21" s="5">
+      <c r="E21" s="1">
+        <v>0</v>
+      </c>
+      <c r="F21" s="1">
         <v>1.5793213512592963</v>
       </c>
-      <c r="G21" s="5">
-        <v>0</v>
-      </c>
-      <c r="H21" s="5">
+      <c r="G21" s="1">
+        <v>0</v>
+      </c>
+      <c r="H21" s="1">
         <v>0</v>
       </c>
       <c r="I21" s="6">
         <v>2.1943095310840208</v>
       </c>
-    </row>
-    <row r="22" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A22" s="4" t="s">
+      <c r="J21" s="1">
+        <f t="shared" ref="J21:J23" si="0">I21/$I$28</f>
+        <v>0.18031830678315613</v>
+      </c>
+    </row>
+    <row r="22" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A22" s="5" t="s">
         <v>236</v>
       </c>
-      <c r="B22" s="5" t="s">
+      <c r="B22" s="1" t="s">
         <v>236</v>
       </c>
-      <c r="C22" s="5">
-        <v>0</v>
-      </c>
-      <c r="D22" s="5">
-        <v>0</v>
-      </c>
-      <c r="E22" s="5">
+      <c r="C22" s="1">
+        <v>0</v>
+      </c>
+      <c r="D22" s="1">
+        <v>0</v>
+      </c>
+      <c r="E22" s="1">
         <v>0.35777816114920324</v>
       </c>
-      <c r="F22" s="5">
-        <v>0</v>
-      </c>
-      <c r="G22" s="5">
+      <c r="F22" s="1">
+        <v>0</v>
+      </c>
+      <c r="G22" s="1">
         <v>0.21013502854748911</v>
       </c>
-      <c r="H22" s="5">
+      <c r="H22" s="1">
         <v>0</v>
       </c>
       <c r="I22" s="6">
         <v>0.56791318969669236</v>
       </c>
-    </row>
-    <row r="23" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A23" s="4" t="s">
+      <c r="J22" s="1">
+        <f t="shared" si="0"/>
+        <v>4.6668504746155519E-2</v>
+      </c>
+    </row>
+    <row r="23" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A23" s="5" t="s">
         <v>237</v>
       </c>
-      <c r="B23" s="5" t="s">
+      <c r="B23" s="1" t="s">
         <v>237</v>
       </c>
-      <c r="C23" s="5">
-        <v>0</v>
-      </c>
-      <c r="D23" s="5">
+      <c r="C23" s="1">
+        <v>0</v>
+      </c>
+      <c r="D23" s="1">
         <v>0.61498817982472431</v>
       </c>
-      <c r="E23" s="5">
+      <c r="E23" s="1">
         <v>0.35777816114920324</v>
       </c>
-      <c r="F23" s="5">
-        <v>0</v>
-      </c>
-      <c r="G23" s="5">
-        <v>0</v>
-      </c>
-      <c r="H23" s="5">
+      <c r="F23" s="1">
+        <v>0</v>
+      </c>
+      <c r="G23" s="1">
+        <v>0</v>
+      </c>
+      <c r="H23" s="1">
         <v>0</v>
       </c>
       <c r="I23" s="6">
         <v>0.97276634097392756</v>
       </c>
-    </row>
-    <row r="24" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A24" s="4"/>
-      <c r="B24" s="5"/>
-      <c r="C24" s="5">
-        <v>0</v>
-      </c>
-      <c r="D24" s="5">
-        <v>0</v>
-      </c>
-      <c r="E24" s="5">
-        <v>0</v>
-      </c>
-      <c r="F24" s="5">
-        <v>0</v>
-      </c>
-      <c r="G24" s="5">
-        <v>0</v>
-      </c>
-      <c r="H24" s="5">
+      <c r="J23" s="1">
+        <f t="shared" si="0"/>
+        <v>7.9937482390376818E-2</v>
+      </c>
+    </row>
+    <row r="24" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A24" s="5"/>
+      <c r="C24" s="1">
+        <v>0</v>
+      </c>
+      <c r="D24" s="1">
+        <v>0</v>
+      </c>
+      <c r="E24" s="1">
+        <v>0</v>
+      </c>
+      <c r="F24" s="1">
+        <v>0</v>
+      </c>
+      <c r="G24" s="1">
+        <v>0</v>
+      </c>
+      <c r="H24" s="1">
         <v>0</v>
       </c>
       <c r="I24" s="6">
         <v>0</v>
       </c>
     </row>
-    <row r="25" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A25" s="4"/>
-      <c r="B25" s="5"/>
-      <c r="C25" s="5">
-        <v>0</v>
-      </c>
-      <c r="D25" s="5">
-        <v>0</v>
-      </c>
-      <c r="E25" s="5">
-        <v>0</v>
-      </c>
-      <c r="F25" s="5">
-        <v>0</v>
-      </c>
-      <c r="G25" s="5">
-        <v>0</v>
-      </c>
-      <c r="H25" s="5">
+    <row r="25" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A25" s="5"/>
+      <c r="C25" s="1">
+        <v>0</v>
+      </c>
+      <c r="D25" s="1">
+        <v>0</v>
+      </c>
+      <c r="E25" s="1">
+        <v>0</v>
+      </c>
+      <c r="F25" s="1">
+        <v>0</v>
+      </c>
+      <c r="G25" s="1">
+        <v>0</v>
+      </c>
+      <c r="H25" s="1">
         <v>0</v>
       </c>
       <c r="I25" s="6">
         <v>0</v>
       </c>
     </row>
-    <row r="26" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A26" s="4"/>
-      <c r="B26" s="5"/>
-      <c r="C26" s="5">
-        <v>0</v>
-      </c>
-      <c r="D26" s="5">
-        <v>0</v>
-      </c>
-      <c r="E26" s="5">
-        <v>0</v>
-      </c>
-      <c r="F26" s="5">
-        <v>0</v>
-      </c>
-      <c r="G26" s="5">
-        <v>0</v>
-      </c>
-      <c r="H26" s="5">
+    <row r="26" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A26" s="5"/>
+      <c r="C26" s="1">
+        <v>0</v>
+      </c>
+      <c r="D26" s="1">
+        <v>0</v>
+      </c>
+      <c r="E26" s="1">
+        <v>0</v>
+      </c>
+      <c r="F26" s="1">
+        <v>0</v>
+      </c>
+      <c r="G26" s="1">
+        <v>0</v>
+      </c>
+      <c r="H26" s="1">
         <v>0</v>
       </c>
       <c r="I26" s="6">
         <v>0</v>
       </c>
     </row>
-    <row r="27" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A27" s="4"/>
-      <c r="B27" s="5"/>
-      <c r="C27" s="5">
-        <v>0</v>
-      </c>
-      <c r="D27" s="5">
-        <v>0</v>
-      </c>
-      <c r="E27" s="5">
-        <v>0</v>
-      </c>
-      <c r="F27" s="5">
-        <v>0</v>
-      </c>
-      <c r="G27" s="5">
-        <v>0</v>
-      </c>
-      <c r="H27" s="5">
+    <row r="27" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A27" s="5"/>
+      <c r="C27" s="1">
+        <v>0</v>
+      </c>
+      <c r="D27" s="1">
+        <v>0</v>
+      </c>
+      <c r="E27" s="1">
+        <v>0</v>
+      </c>
+      <c r="F27" s="1">
+        <v>0</v>
+      </c>
+      <c r="G27" s="1">
+        <v>0</v>
+      </c>
+      <c r="H27" s="1">
         <v>0</v>
       </c>
       <c r="I27" s="6">
         <v>0</v>
       </c>
     </row>
-    <row r="28" spans="1:9" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="28" spans="1:10" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A28" s="7"/>
       <c r="B28" s="8"/>
       <c r="C28" s="8">
@@ -1604,6 +1647,107 @@
       <c r="I28" s="9">
         <v>12.16908904165129</v>
       </c>
+    </row>
+    <row r="29" spans="1:10" ht="15" thickBot="1" x14ac:dyDescent="0.35"/>
+    <row r="30" spans="1:10" ht="72" x14ac:dyDescent="0.3">
+      <c r="A30" s="2"/>
+      <c r="B30" s="3"/>
+      <c r="C30" s="3" t="s">
+        <v>224</v>
+      </c>
+      <c r="D30" s="3" t="s">
+        <v>225</v>
+      </c>
+      <c r="E30" s="3" t="s">
+        <v>233</v>
+      </c>
+      <c r="F30" s="3" t="s">
+        <v>234</v>
+      </c>
+      <c r="G30" s="3" t="s">
+        <v>228</v>
+      </c>
+      <c r="H30" s="3" t="s">
+        <v>229</v>
+      </c>
+      <c r="I30" s="4" t="s">
+        <v>230</v>
+      </c>
+    </row>
+    <row r="31" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A31" s="5" t="s">
+        <v>235</v>
+      </c>
+      <c r="C31" s="1">
+        <v>1</v>
+      </c>
+      <c r="H31" s="1">
+        <v>1</v>
+      </c>
+      <c r="I31" s="6"/>
+    </row>
+    <row r="32" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A32" s="5" t="s">
+        <v>0</v>
+      </c>
+      <c r="D32" s="1" t="s">
+        <v>239</v>
+      </c>
+      <c r="F32" s="1">
+        <v>1</v>
+      </c>
+      <c r="I32" s="6"/>
+    </row>
+    <row r="33" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A33" s="5" t="s">
+        <v>236</v>
+      </c>
+      <c r="E33" s="1" t="s">
+        <v>239</v>
+      </c>
+      <c r="G33" s="1">
+        <v>1</v>
+      </c>
+      <c r="I33" s="6"/>
+    </row>
+    <row r="34" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A34" s="5" t="s">
+        <v>237</v>
+      </c>
+      <c r="D34" s="1" t="s">
+        <v>239</v>
+      </c>
+      <c r="E34" s="1" t="s">
+        <v>239</v>
+      </c>
+      <c r="I34" s="6"/>
+    </row>
+    <row r="35" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A35" s="5"/>
+      <c r="I35" s="6"/>
+    </row>
+    <row r="36" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A36" s="5"/>
+      <c r="I36" s="6"/>
+    </row>
+    <row r="37" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A37" s="5"/>
+      <c r="I37" s="6"/>
+    </row>
+    <row r="38" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A38" s="5"/>
+      <c r="I38" s="6"/>
+    </row>
+    <row r="39" spans="1:9" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A39" s="7"/>
+      <c r="B39" s="8"/>
+      <c r="C39" s="8"/>
+      <c r="D39" s="8"/>
+      <c r="E39" s="8"/>
+      <c r="F39" s="8"/>
+      <c r="G39" s="8"/>
+      <c r="H39" s="8"/>
+      <c r="I39" s="9"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -1616,7 +1760,7 @@
   <dimension ref="A1:B5"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="62.77734375" customWidth="1"/>
+    <col min="1" max="1" width="31.44140625" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.3">
@@ -4057,21 +4201,21 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<TemplafyTemplateConfiguration><![CDATA[{"transformationConfigurations":[],"templateName":"blankspreadsheet","templateDescription":"","enableDocumentContentUpdater":false,"version":"2.0"}]]></TemplafyTemplateConfiguration>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <TemplafyFormConfiguration><![CDATA[{"formFields":[],"formDataEntries":[]}]]></TemplafyFormConfiguration>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<TemplafyTemplateConfiguration><![CDATA[{"transformationConfigurations":[],"templateName":"blankspreadsheet","templateDescription":"","enableDocumentContentUpdater":false,"version":"2.0"}]]></TemplafyTemplateConfiguration>
-</file>
-
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{613AEFFE-C095-42A7-A0AC-5564FFC1D197}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{7408D0D6-C97A-426B-8466-DDDAA7A3F420}">
   <ds:schemaRefs/>
 </ds:datastoreItem>
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{7408D0D6-C97A-426B-8466-DDDAA7A3F420}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{613AEFFE-C095-42A7-A0AC-5564FFC1D197}">
   <ds:schemaRefs/>
 </ds:datastoreItem>
 </file>
</xml_diff>